<commit_message>
update (comit safadfo kkkk)
</commit_message>
<xml_diff>
--- a/data/tabela_combinada_final.xlsx
+++ b/data/tabela_combinada_final.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\OneDrive\Documentos\TP\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\OneDrive\Documentos\D.comercial\dashboard streamlit\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F568CF-0266-4EC8-A481-694E26B55029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC35640-23F6-4E47-A92D-2076D7937882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="382">
   <si>
     <t>Nome do Participante</t>
   </si>
@@ -114,9 +114,6 @@
     <t>05 horas</t>
   </si>
   <si>
-    <t>Sim, lua crescente</t>
-  </si>
-  <si>
     <t>Sim</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
     <t>5 a 8 horas</t>
   </si>
   <si>
-    <t>Sim, lua nova</t>
-  </si>
-  <si>
     <t>Bagre, tainha, robalo, pescada</t>
   </si>
   <si>
@@ -201,9 +195,6 @@
     <t>4 horas</t>
   </si>
   <si>
-    <t>Não, depende da maré</t>
-  </si>
-  <si>
     <t>Robalo e pescada</t>
   </si>
   <si>
@@ -333,9 +324,6 @@
     <t>12 horas</t>
   </si>
   <si>
-    <t>Sim, quarto crescente</t>
-  </si>
-  <si>
     <t>Pescada, Camurim, Bagre</t>
   </si>
   <si>
@@ -435,9 +423,6 @@
     <t>5 a 7 dias</t>
   </si>
   <si>
-    <t>Sim, lua escura</t>
-  </si>
-  <si>
     <t>Bagre, pescadinha e etc.</t>
   </si>
   <si>
@@ -471,9 +456,6 @@
     <t>2 dias</t>
   </si>
   <si>
-    <t>sim, lua minguante</t>
-  </si>
-  <si>
     <t>Robalo e camurim</t>
   </si>
   <si>
@@ -558,9 +540,6 @@
     <t>Até 2 dias</t>
   </si>
   <si>
-    <t>Sim, lua cheia</t>
-  </si>
-  <si>
     <t>Robalo, carapeba, bagre</t>
   </si>
   <si>
@@ -624,9 +603,6 @@
     <t>De 3 a 4 horas</t>
   </si>
   <si>
-    <t>Sim, maré, claridade</t>
-  </si>
-  <si>
     <t>Bagre, camurim, carapeba</t>
   </si>
   <si>
@@ -657,9 +633,6 @@
     <t xml:space="preserve">Sim, às 22:00 hs </t>
   </si>
   <si>
-    <t>Sim, lua minguante</t>
-  </si>
-  <si>
     <t>Bagre, camurim , pescadinha, carapeba</t>
   </si>
   <si>
@@ -741,9 +714,6 @@
     <t>6 horas</t>
   </si>
   <si>
-    <t>Sim, lua minguante e crescente</t>
-  </si>
-  <si>
     <t>Bagre, pescada e arraia</t>
   </si>
   <si>
@@ -894,9 +864,6 @@
     <t>Caçoeira</t>
   </si>
   <si>
-    <t>Sim, sem claridade da lua</t>
-  </si>
-  <si>
     <t>Camurim, pescada amarela e branca, coró, bagre e outros</t>
   </si>
   <si>
@@ -966,9 +933,6 @@
     <t>De 10 a 12 horas</t>
   </si>
   <si>
-    <t>Sim, lua crescente e minguante</t>
-  </si>
-  <si>
     <t>Bagre, curuca, pescada amarela e branca, serra, pilombeta, arraia</t>
   </si>
   <si>
@@ -1128,9 +1092,6 @@
     <t>Sim, por volta de 06:00 hs</t>
   </si>
   <si>
-    <t>Sim, minguante</t>
-  </si>
-  <si>
     <t>Bagre, pescadinha, curuca, coro</t>
   </si>
   <si>
@@ -1143,9 +1104,6 @@
     <t>Sim, dentro do rio</t>
   </si>
   <si>
-    <t>Sim, quarto minguante</t>
-  </si>
-  <si>
     <t>Pescada, tainha, bagre, capeba, curuca, barbudo</t>
   </si>
   <si>
@@ -1198,6 +1156,21 @@
   </si>
   <si>
     <t>Raimundo Rodrigues Oliveira</t>
+  </si>
+  <si>
+    <t>lua crescente</t>
+  </si>
+  <si>
+    <t>lua nova</t>
+  </si>
+  <si>
+    <t>lua minguante</t>
+  </si>
+  <si>
+    <t>lua cheia</t>
+  </si>
+  <si>
+    <t>lua escura</t>
   </si>
 </sst>
 </file>
@@ -1676,295 +1649,295 @@
         <v>28</v>
       </c>
       <c r="N2" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O2" t="s">
         <v>21</v>
       </c>
       <c r="P2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" t="s">
         <v>30</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>66</v>
       </c>
       <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
         <v>33</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>34</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>36</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>37</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>38</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>39</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>40</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>41</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>42</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
+        <v>378</v>
+      </c>
+      <c r="O3" t="s">
         <v>43</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>44</v>
       </c>
-      <c r="O3" t="s">
-        <v>45</v>
-      </c>
-      <c r="P3" t="s">
-        <v>46</v>
-      </c>
       <c r="Q3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B4">
         <v>65</v>
       </c>
       <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
         <v>48</v>
-      </c>
-      <c r="D4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" t="s">
-        <v>50</v>
       </c>
       <c r="F4" t="s">
         <v>21</v>
       </c>
       <c r="G4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" t="s">
         <v>51</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>52</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>53</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>54</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
         <v>55</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" t="s">
         <v>56</v>
       </c>
-      <c r="M4" t="s">
+      <c r="P4" t="s">
         <v>57</v>
       </c>
-      <c r="N4" t="s">
-        <v>58</v>
-      </c>
-      <c r="O4" t="s">
-        <v>59</v>
-      </c>
-      <c r="P4" t="s">
-        <v>60</v>
-      </c>
       <c r="Q4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B5">
         <v>54</v>
       </c>
       <c r="C5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
         <v>62</v>
       </c>
-      <c r="D5" t="s">
+      <c r="I5" t="s">
         <v>63</v>
       </c>
-      <c r="E5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="J5" t="s">
         <v>64</v>
       </c>
-      <c r="H5" t="s">
+      <c r="K5" t="s">
         <v>65</v>
       </c>
-      <c r="I5" t="s">
+      <c r="L5" t="s">
         <v>66</v>
       </c>
-      <c r="J5" t="s">
+      <c r="M5" t="s">
         <v>67</v>
       </c>
-      <c r="K5" t="s">
+      <c r="N5" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" t="s">
         <v>68</v>
       </c>
-      <c r="L5" t="s">
-        <v>69</v>
-      </c>
-      <c r="M5" t="s">
-        <v>70</v>
-      </c>
-      <c r="N5" t="s">
-        <v>46</v>
-      </c>
-      <c r="O5" t="s">
-        <v>71</v>
-      </c>
       <c r="P5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Q5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B6">
         <v>62</v>
       </c>
       <c r="C6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" t="s">
         <v>73</v>
-      </c>
-      <c r="D6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" t="s">
-        <v>74</v>
-      </c>
-      <c r="F6" t="s">
-        <v>75</v>
-      </c>
-      <c r="G6" t="s">
-        <v>76</v>
       </c>
       <c r="H6" t="s">
         <v>23</v>
       </c>
       <c r="I6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J6" t="s">
+        <v>74</v>
+      </c>
+      <c r="K6" t="s">
+        <v>75</v>
+      </c>
+      <c r="L6" t="s">
+        <v>76</v>
+      </c>
+      <c r="M6" t="s">
         <v>77</v>
       </c>
-      <c r="K6" t="s">
+      <c r="N6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O6" t="s">
         <v>78</v>
       </c>
-      <c r="L6" t="s">
-        <v>79</v>
-      </c>
-      <c r="M6" t="s">
-        <v>80</v>
-      </c>
-      <c r="N6" t="s">
-        <v>46</v>
-      </c>
-      <c r="O6" t="s">
-        <v>81</v>
-      </c>
       <c r="P6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Q6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B7">
         <v>71</v>
       </c>
       <c r="C7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" t="s">
         <v>83</v>
       </c>
-      <c r="D7" t="s">
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="E7" t="s">
+      <c r="I7" t="s">
         <v>85</v>
-      </c>
-      <c r="F7" t="s">
-        <v>86</v>
-      </c>
-      <c r="G7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" t="s">
-        <v>88</v>
       </c>
       <c r="J7" t="s">
         <v>25</v>
       </c>
       <c r="K7" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" t="s">
+        <v>87</v>
+      </c>
+      <c r="M7" t="s">
+        <v>88</v>
+      </c>
+      <c r="N7" t="s">
+        <v>378</v>
+      </c>
+      <c r="O7" t="s">
         <v>89</v>
       </c>
-      <c r="L7" t="s">
+      <c r="P7" t="s">
         <v>90</v>
       </c>
-      <c r="M7" t="s">
-        <v>91</v>
-      </c>
-      <c r="N7" t="s">
-        <v>44</v>
-      </c>
-      <c r="O7" t="s">
-        <v>92</v>
-      </c>
-      <c r="P7" t="s">
-        <v>93</v>
-      </c>
       <c r="Q7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B8">
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
         <v>20</v>
@@ -1973,7 +1946,7 @@
         <v>21</v>
       </c>
       <c r="G8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H8" t="s">
         <v>23</v>
@@ -1982,42 +1955,42 @@
         <v>24</v>
       </c>
       <c r="J8" t="s">
+        <v>95</v>
+      </c>
+      <c r="K8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L8" t="s">
+        <v>97</v>
+      </c>
+      <c r="M8" t="s">
         <v>98</v>
       </c>
-      <c r="K8" t="s">
+      <c r="N8" t="s">
+        <v>377</v>
+      </c>
+      <c r="O8" t="s">
         <v>99</v>
       </c>
-      <c r="L8" t="s">
-        <v>100</v>
-      </c>
-      <c r="M8" t="s">
-        <v>101</v>
-      </c>
-      <c r="N8" t="s">
-        <v>102</v>
-      </c>
-      <c r="O8" t="s">
-        <v>103</v>
-      </c>
       <c r="P8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B9">
         <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E9" t="s">
         <v>21</v>
@@ -2026,263 +1999,263 @@
         <v>21</v>
       </c>
       <c r="G9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H9" t="s">
+        <v>104</v>
+      </c>
+      <c r="I9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" t="s">
+        <v>106</v>
+      </c>
+      <c r="K9" t="s">
         <v>107</v>
       </c>
-      <c r="H9" t="s">
+      <c r="L9" t="s">
         <v>108</v>
       </c>
-      <c r="I9" t="s">
+      <c r="M9" t="s">
         <v>109</v>
       </c>
-      <c r="J9" t="s">
+      <c r="N9" t="s">
+        <v>44</v>
+      </c>
+      <c r="O9" t="s">
         <v>110</v>
       </c>
-      <c r="K9" t="s">
-        <v>111</v>
-      </c>
-      <c r="L9" t="s">
-        <v>112</v>
-      </c>
-      <c r="M9" t="s">
-        <v>113</v>
-      </c>
-      <c r="N9" t="s">
-        <v>46</v>
-      </c>
-      <c r="O9" t="s">
-        <v>114</v>
-      </c>
       <c r="P9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B10">
         <v>58</v>
       </c>
       <c r="C10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F10" t="s">
+        <v>115</v>
+      </c>
+      <c r="G10" t="s">
         <v>116</v>
       </c>
-      <c r="D10" t="s">
+      <c r="H10" t="s">
         <v>117</v>
       </c>
-      <c r="E10" t="s">
+      <c r="I10" t="s">
         <v>118</v>
       </c>
-      <c r="F10" t="s">
+      <c r="J10" t="s">
         <v>119</v>
       </c>
-      <c r="G10" t="s">
+      <c r="K10" t="s">
         <v>120</v>
       </c>
-      <c r="H10" t="s">
+      <c r="L10" t="s">
         <v>121</v>
       </c>
-      <c r="I10" t="s">
+      <c r="M10" t="s">
         <v>122</v>
       </c>
-      <c r="J10" t="s">
+      <c r="N10" t="s">
+        <v>377</v>
+      </c>
+      <c r="O10" t="s">
         <v>123</v>
       </c>
-      <c r="K10" t="s">
+      <c r="P10" t="s">
         <v>124</v>
       </c>
-      <c r="L10" t="s">
+      <c r="Q10" t="s">
         <v>125</v>
-      </c>
-      <c r="M10" t="s">
-        <v>126</v>
-      </c>
-      <c r="N10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O10" t="s">
-        <v>127</v>
-      </c>
-      <c r="P10" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B11">
         <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F11" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G11" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H11" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I11" t="s">
         <v>24</v>
       </c>
       <c r="J11" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K11" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L11" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M11" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N11" t="s">
-        <v>136</v>
+        <v>378</v>
       </c>
       <c r="O11" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="P11" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="Q11" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B12">
         <v>55</v>
       </c>
       <c r="C12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" t="s">
+        <v>136</v>
+      </c>
+      <c r="G12" t="s">
+        <v>137</v>
+      </c>
+      <c r="H12" t="s">
+        <v>138</v>
+      </c>
+      <c r="I12" t="s">
+        <v>118</v>
+      </c>
+      <c r="J12" t="s">
         <v>139</v>
       </c>
-      <c r="D12" t="s">
+      <c r="K12" t="s">
         <v>140</v>
       </c>
-      <c r="E12" t="s">
-        <v>132</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="L12" t="s">
         <v>141</v>
       </c>
-      <c r="G12" t="s">
+      <c r="M12" t="s">
         <v>142</v>
       </c>
-      <c r="H12" t="s">
+      <c r="N12" t="s">
+        <v>379</v>
+      </c>
+      <c r="O12" t="s">
         <v>143</v>
       </c>
-      <c r="I12" t="s">
-        <v>122</v>
-      </c>
-      <c r="J12" t="s">
-        <v>144</v>
-      </c>
-      <c r="K12" t="s">
-        <v>145</v>
-      </c>
-      <c r="L12" t="s">
-        <v>146</v>
-      </c>
-      <c r="M12" t="s">
-        <v>147</v>
-      </c>
-      <c r="N12" t="s">
-        <v>148</v>
-      </c>
-      <c r="O12" t="s">
-        <v>149</v>
-      </c>
       <c r="P12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q12" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B13">
         <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D13" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E13" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F13" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H13" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I13" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K13" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="L13" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="M13" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="N13" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O13" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="P13" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B14">
         <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D14" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E14" t="s">
         <v>21</v>
@@ -2291,51 +2264,51 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H14" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I14" t="s">
         <v>24</v>
       </c>
       <c r="J14" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K14" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L14" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="M14" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="N14" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O14" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="P14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q14" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B15">
         <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E15" t="s">
         <v>21</v>
@@ -2344,275 +2317,275 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H15" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J15" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="K15" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="L15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M15" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="N15" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O15" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="P15" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q15" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B16">
         <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D16" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E16" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F16" t="s">
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="H16" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I16" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="J16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K16" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="L16" t="s">
+        <v>121</v>
+      </c>
+      <c r="M16" t="s">
+        <v>38</v>
+      </c>
+      <c r="N16" t="s">
+        <v>379</v>
+      </c>
+      <c r="O16" t="s">
+        <v>163</v>
+      </c>
+      <c r="P16" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q16" t="s">
         <v>125</v>
-      </c>
-      <c r="M16" t="s">
-        <v>39</v>
-      </c>
-      <c r="N16" t="s">
-        <v>148</v>
-      </c>
-      <c r="O16" t="s">
-        <v>169</v>
-      </c>
-      <c r="P16" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B17">
         <v>46</v>
       </c>
       <c r="C17" t="s">
+        <v>165</v>
+      </c>
+      <c r="D17" t="s">
+        <v>166</v>
+      </c>
+      <c r="E17" t="s">
+        <v>167</v>
+      </c>
+      <c r="F17" t="s">
+        <v>115</v>
+      </c>
+      <c r="G17" t="s">
+        <v>168</v>
+      </c>
+      <c r="H17" t="s">
+        <v>138</v>
+      </c>
+      <c r="I17" t="s">
+        <v>169</v>
+      </c>
+      <c r="J17" t="s">
+        <v>66</v>
+      </c>
+      <c r="K17" t="s">
+        <v>129</v>
+      </c>
+      <c r="L17" t="s">
+        <v>119</v>
+      </c>
+      <c r="M17" t="s">
+        <v>170</v>
+      </c>
+      <c r="N17" t="s">
+        <v>380</v>
+      </c>
+      <c r="O17" t="s">
         <v>171</v>
       </c>
-      <c r="D17" t="s">
-        <v>172</v>
-      </c>
-      <c r="E17" t="s">
-        <v>173</v>
-      </c>
-      <c r="F17" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" t="s">
-        <v>174</v>
-      </c>
-      <c r="H17" t="s">
-        <v>143</v>
-      </c>
-      <c r="I17" t="s">
-        <v>175</v>
-      </c>
-      <c r="J17" t="s">
-        <v>69</v>
-      </c>
-      <c r="K17" t="s">
-        <v>133</v>
-      </c>
-      <c r="L17" t="s">
-        <v>123</v>
-      </c>
-      <c r="M17" t="s">
-        <v>176</v>
-      </c>
-      <c r="N17" t="s">
-        <v>177</v>
-      </c>
-      <c r="O17" t="s">
-        <v>178</v>
-      </c>
       <c r="P17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q17" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="B18">
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D18" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="E18" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F18" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G18" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
       </c>
       <c r="J18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="K18" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="L18" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="N18" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O18" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="P18" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q18" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="B19">
         <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D19" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E19" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F19" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G19" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H19" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I19" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="J19" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="K19" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L19" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="M19" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="N19" t="s">
-        <v>44</v>
+        <v>378</v>
       </c>
       <c r="O19" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="P19" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="Q19" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="B20">
         <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D20" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="E20" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F20" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G20" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H20" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I20" t="s">
         <v>24</v>
@@ -2621,410 +2594,410 @@
         <v>25</v>
       </c>
       <c r="K20" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="L20" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M20" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="N20" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O20" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P20" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B21">
         <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D21" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="E21" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F21" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G21" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="H21" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J21" t="s">
         <v>25</v>
       </c>
       <c r="K21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="L21" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="M21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="N21" t="s">
-        <v>199</v>
+        <v>380</v>
       </c>
       <c r="O21" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="P21" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q21" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B22">
         <v>56</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D22" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="E22" t="s">
         <v>21</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G22" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H22" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J22" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="K22" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="L22" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="M22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="N22" t="s">
-        <v>136</v>
+        <v>378</v>
       </c>
       <c r="O22" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="P22" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="Q22" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B23">
         <v>62</v>
       </c>
       <c r="C23" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D23" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E23" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F23" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G23" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="H23" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I23" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="J23" t="s">
         <v>25</v>
       </c>
       <c r="K23" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="L23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M23" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="N23" t="s">
-        <v>210</v>
+        <v>379</v>
       </c>
       <c r="O23" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="P23" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="B24">
         <v>63</v>
       </c>
       <c r="C24" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D24" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E24" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="F24" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="G24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H24" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I24" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J24" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="K24" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="L24" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="M24" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="N24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O24" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="P24" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q24" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B25">
         <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D25" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="E25" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="F25" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G25" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H25" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I25" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="J25" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="K25" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="L25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M25" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="N25" t="s">
-        <v>177</v>
+        <v>380</v>
       </c>
       <c r="O25" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="P25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q25" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="B26">
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="D26" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="E26" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="F26" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G26" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="H26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I26" t="s">
         <v>24</v>
       </c>
       <c r="J26" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="K26" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="L26" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="M26" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="N26" t="s">
-        <v>136</v>
+        <v>378</v>
       </c>
       <c r="O26" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="P26" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q26" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="B27">
         <v>53</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D27" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="E27" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F27" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G27" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="H27" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I27" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="J27" t="s">
         <v>25</v>
       </c>
       <c r="K27" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="L27" t="s">
         <v>21</v>
       </c>
       <c r="M27" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="N27" t="s">
-        <v>238</v>
+        <v>379</v>
       </c>
       <c r="O27" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="P27" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q27" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="B28">
         <v>51</v>
       </c>
       <c r="C28" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D28" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="E28" t="s">
         <v>21</v>
@@ -3033,328 +3006,325 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H28" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I28" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="J28" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K28" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L28" t="s">
+        <v>121</v>
+      </c>
+      <c r="M28" t="s">
+        <v>191</v>
+      </c>
+      <c r="N28" t="s">
+        <v>377</v>
+      </c>
+      <c r="O28" t="s">
+        <v>234</v>
+      </c>
+      <c r="P28" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q28" t="s">
         <v>125</v>
-      </c>
-      <c r="M28" t="s">
-        <v>198</v>
-      </c>
-      <c r="N28" t="s">
-        <v>29</v>
-      </c>
-      <c r="O28" t="s">
-        <v>244</v>
-      </c>
-      <c r="P28" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="B29">
         <v>49</v>
       </c>
       <c r="C29" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D29" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="E29" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="F29" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="G29" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="H29" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I29" t="s">
+        <v>232</v>
+      </c>
+      <c r="J29" t="s">
+        <v>239</v>
+      </c>
+      <c r="K29" t="s">
+        <v>240</v>
+      </c>
+      <c r="L29" t="s">
+        <v>233</v>
+      </c>
+      <c r="M29" t="s">
+        <v>241</v>
+      </c>
+      <c r="N29" t="s">
+        <v>378</v>
+      </c>
+      <c r="O29" t="s">
         <v>242</v>
       </c>
-      <c r="J29" t="s">
-        <v>249</v>
-      </c>
-      <c r="K29" t="s">
-        <v>250</v>
-      </c>
-      <c r="L29" t="s">
+      <c r="P29" t="s">
         <v>243</v>
       </c>
-      <c r="M29" t="s">
-        <v>251</v>
-      </c>
-      <c r="N29" t="s">
-        <v>44</v>
-      </c>
-      <c r="O29" t="s">
-        <v>252</v>
-      </c>
-      <c r="P29" t="s">
-        <v>253</v>
-      </c>
       <c r="Q29" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="B30">
         <v>74</v>
       </c>
       <c r="C30" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="D30" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="E30" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="F30" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G30" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="H30" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I30" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="J30" t="s">
+        <v>239</v>
+      </c>
+      <c r="K30" t="s">
+        <v>44</v>
+      </c>
+      <c r="L30" t="s">
         <v>249</v>
       </c>
-      <c r="K30" t="s">
-        <v>46</v>
-      </c>
-      <c r="L30" t="s">
-        <v>259</v>
-      </c>
       <c r="M30" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="N30" t="s">
-        <v>136</v>
+        <v>378</v>
       </c>
       <c r="O30" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="P30" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Q30" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="B31">
         <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D31" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E31" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F31" t="s">
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H31" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I31" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J31" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="K31" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="L31" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="M31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N31" t="s">
-        <v>199</v>
+        <v>380</v>
       </c>
       <c r="O31" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="P31" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q31" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="B32">
         <v>57</v>
       </c>
       <c r="C32" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D32" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E32" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F32" t="s">
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="H32" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I32" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="J32" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="K32" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="L32" t="s">
+        <v>121</v>
+      </c>
+      <c r="M32" t="s">
+        <v>260</v>
+      </c>
+      <c r="O32" t="s">
+        <v>261</v>
+      </c>
+      <c r="P32" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q32" t="s">
         <v>125</v>
-      </c>
-      <c r="M32" t="s">
-        <v>270</v>
-      </c>
-      <c r="N32" t="s">
-        <v>30</v>
-      </c>
-      <c r="O32" t="s">
-        <v>271</v>
-      </c>
-      <c r="P32" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="B33">
         <v>37</v>
       </c>
       <c r="C33" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D33" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F33" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G33" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="H33" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I33" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="J33" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="K33" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="L33" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="M33" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="N33" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O33" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="P33" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q33" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="B34">
         <v>30</v>
       </c>
       <c r="C34" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
       </c>
       <c r="E34" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F34" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="G34" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="H34" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I34" t="s">
         <v>24</v>
@@ -3363,323 +3333,323 @@
         <v>21</v>
       </c>
       <c r="K34" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L34" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="M34" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="N34" t="s">
-        <v>177</v>
+        <v>380</v>
       </c>
       <c r="O34" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="P34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Q34" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="B35">
         <v>44</v>
       </c>
       <c r="C35" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="D35" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="E35" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F35" t="s">
         <v>21</v>
       </c>
       <c r="G35" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H35" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I35" t="s">
         <v>24</v>
       </c>
       <c r="J35" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K35" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L35" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M35" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="N35" t="s">
-        <v>289</v>
+        <v>378</v>
       </c>
       <c r="O35" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="P35" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="Q35" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="B36">
         <v>56</v>
       </c>
       <c r="C36" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D36" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E36" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="F36" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G36" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I36" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="J36" t="s">
         <v>25</v>
       </c>
       <c r="K36" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="L36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M36" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="N36" t="s">
-        <v>102</v>
+        <v>377</v>
       </c>
       <c r="O36" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="P36" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="Q36" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="B37">
         <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D37" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E37" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="F37" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G37" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H37" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I37" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="J37" t="s">
         <v>25</v>
       </c>
       <c r="K37" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="L37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M37" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="N37" t="s">
-        <v>102</v>
+        <v>377</v>
       </c>
       <c r="O37" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="P37" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="Q37" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="C38" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D38" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E38" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="F38" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G38" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H38" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I38" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="J38" t="s">
         <v>25</v>
       </c>
       <c r="K38" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="L38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M38" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="N38" t="s">
-        <v>102</v>
+        <v>377</v>
       </c>
       <c r="O38" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="P38" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="Q38" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="B39">
         <v>34</v>
       </c>
       <c r="Q39" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="B40">
         <v>73</v>
       </c>
       <c r="Q40" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="B41">
         <v>44</v>
       </c>
       <c r="C41" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D41" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="E41" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="F41" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="G41" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="H41" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I41" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="J41" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="K41" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="L41" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="M41" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="N41" t="s">
-        <v>313</v>
+        <v>377</v>
       </c>
       <c r="O41" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="P41" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Q41" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="B42">
         <v>52</v>
       </c>
       <c r="C42" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D42" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E42" t="s">
         <v>21</v>
@@ -3688,820 +3658,814 @@
         <v>21</v>
       </c>
       <c r="G42" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H42" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I42" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J42" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="K42" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L42" t="s">
         <v>21</v>
       </c>
       <c r="M42" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="N42" t="s">
-        <v>29</v>
+        <v>377</v>
       </c>
       <c r="O42" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="P42" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q42" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="B43">
         <v>45</v>
       </c>
       <c r="C43" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D43" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="E43" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F43" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="G43" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="H43" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I43" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="J43" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="K43" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L43" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="M43" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="N43" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O43" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="P43" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q43" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="B44">
         <v>32</v>
       </c>
       <c r="C44" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="D44" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="E44" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="F44" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="G44" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H44" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I44" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="J44" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K44" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="L44" t="s">
         <v>25</v>
       </c>
       <c r="M44" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="N44" t="s">
-        <v>44</v>
+        <v>378</v>
       </c>
       <c r="O44" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="P44" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q44" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="B45">
         <v>26</v>
       </c>
       <c r="C45" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D45" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="E45" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="F45" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="G45" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="H45" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I45" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="J45" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="K45" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="L45" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="M45" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="N45" t="s">
-        <v>313</v>
+        <v>377</v>
       </c>
       <c r="O45" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="P45" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q45" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="B46">
         <v>55</v>
       </c>
       <c r="C46" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D46" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="E46" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F46" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="G46" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="H46" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I46" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="J46" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="K46" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L46" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="M46" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="N46" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O46" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="P46" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q46" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="B47">
         <v>51</v>
       </c>
       <c r="C47" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="D47" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="E47" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="F47" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G47" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="H47" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I47" t="s">
         <v>24</v>
       </c>
       <c r="J47" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="K47" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L47" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="M47" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="N47" t="s">
-        <v>177</v>
+        <v>380</v>
       </c>
       <c r="O47" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="P47" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q47" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="B48">
         <v>41</v>
       </c>
       <c r="C48" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D48" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="E48" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="F48" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G48" t="s">
+        <v>324</v>
+      </c>
+      <c r="H48" t="s">
+        <v>138</v>
+      </c>
+      <c r="I48" t="s">
+        <v>334</v>
+      </c>
+      <c r="J48" t="s">
+        <v>206</v>
+      </c>
+      <c r="K48" t="s">
+        <v>73</v>
+      </c>
+      <c r="L48" t="s">
+        <v>335</v>
+      </c>
+      <c r="M48" t="s">
         <v>336</v>
       </c>
-      <c r="H48" t="s">
-        <v>143</v>
-      </c>
-      <c r="I48" t="s">
-        <v>346</v>
-      </c>
-      <c r="J48" t="s">
-        <v>215</v>
-      </c>
-      <c r="K48" t="s">
-        <v>76</v>
-      </c>
-      <c r="L48" t="s">
-        <v>347</v>
-      </c>
-      <c r="M48" t="s">
-        <v>348</v>
-      </c>
       <c r="N48" t="s">
-        <v>136</v>
+        <v>381</v>
       </c>
       <c r="O48" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="P48" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="Q48" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="B49">
         <v>45</v>
       </c>
       <c r="C49" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D49" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="E49" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F49" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="G49" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="H49" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I49" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="J49" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="K49" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L49" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="M49" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="N49" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O49" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="P49" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="Q49" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="B50">
         <v>53</v>
       </c>
       <c r="C50" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D50" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E50" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="F50" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G50" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="H50" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I50" t="s">
+        <v>63</v>
+      </c>
+      <c r="J50" t="s">
         <v>66</v>
       </c>
-      <c r="J50" t="s">
-        <v>69</v>
-      </c>
       <c r="K50" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="L50" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="M50" t="s">
-        <v>155</v>
-      </c>
-      <c r="N50" t="s">
-        <v>30</v>
+        <v>149</v>
       </c>
       <c r="O50" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="P50" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q50" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="B51">
         <v>32</v>
       </c>
       <c r="C51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D51" t="s">
         <v>20</v>
       </c>
       <c r="G51" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H51" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="I51" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J51" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="K51" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="L51" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="M51" t="s">
-        <v>113</v>
-      </c>
-      <c r="N51" t="s">
-        <v>30</v>
+        <v>109</v>
       </c>
       <c r="O51" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="P51" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q51" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="B52">
         <v>54</v>
       </c>
       <c r="C52" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D52" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="G52" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="H52" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I52" t="s">
+        <v>334</v>
+      </c>
+      <c r="J52" t="s">
+        <v>76</v>
+      </c>
+      <c r="K52" t="s">
+        <v>354</v>
+      </c>
+      <c r="L52" t="s">
+        <v>119</v>
+      </c>
+      <c r="M52" t="s">
+        <v>109</v>
+      </c>
+      <c r="N52" t="s">
+        <v>379</v>
+      </c>
+      <c r="O52" t="s">
+        <v>355</v>
+      </c>
+      <c r="P52" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q52" t="s">
         <v>346</v>
-      </c>
-      <c r="J52" t="s">
-        <v>79</v>
-      </c>
-      <c r="K52" t="s">
-        <v>366</v>
-      </c>
-      <c r="L52" t="s">
-        <v>123</v>
-      </c>
-      <c r="M52" t="s">
-        <v>113</v>
-      </c>
-      <c r="N52" t="s">
-        <v>367</v>
-      </c>
-      <c r="O52" t="s">
-        <v>368</v>
-      </c>
-      <c r="P52" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q52" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>369</v>
+        <v>356</v>
       </c>
       <c r="B53">
         <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>370</v>
+        <v>357</v>
       </c>
       <c r="D53" t="s">
         <v>20</v>
       </c>
       <c r="G53" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="H53" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="J53" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="K53" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="L53" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M53" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="N53" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="O53" t="s">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="P53" t="s">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="Q53" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>375</v>
+        <v>361</v>
       </c>
       <c r="B54">
         <v>63</v>
       </c>
       <c r="C54" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="D54" t="s">
         <v>20</v>
       </c>
       <c r="G54" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="H54" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I54" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J54" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K54" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L54" t="s">
-        <v>376</v>
+        <v>362</v>
       </c>
       <c r="M54" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="N54" t="s">
-        <v>177</v>
+        <v>380</v>
       </c>
       <c r="O54" t="s">
-        <v>377</v>
+        <v>363</v>
       </c>
       <c r="P54" t="s">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="Q54" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>378</v>
+        <v>364</v>
       </c>
       <c r="B55">
         <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="D55" t="s">
         <v>20</v>
       </c>
       <c r="G55" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H55" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="J55" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K55" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="L55" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M55" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="N55" t="s">
-        <v>44</v>
+        <v>378</v>
       </c>
       <c r="O55" t="s">
-        <v>379</v>
+        <v>365</v>
       </c>
       <c r="P55" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q55" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>380</v>
+        <v>366</v>
       </c>
       <c r="B56">
         <v>41</v>
       </c>
       <c r="C56" t="s">
-        <v>370</v>
+        <v>357</v>
       </c>
       <c r="D56" t="s">
         <v>20</v>
       </c>
       <c r="G56" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="H56" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I56" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J56" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="K56" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="L56" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M56" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="N56" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="O56" t="s">
-        <v>381</v>
+        <v>367</v>
       </c>
       <c r="P56" t="s">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="Q56" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>382</v>
+        <v>368</v>
       </c>
       <c r="B57">
         <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D57" t="s">
-        <v>383</v>
+        <v>369</v>
       </c>
       <c r="E57" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="F57" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G57" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H57" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="J57" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="K57" t="s">
-        <v>385</v>
+        <v>371</v>
       </c>
       <c r="L57" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="M57" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="N57" t="s">
-        <v>102</v>
+        <v>377</v>
       </c>
       <c r="O57" t="s">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="P57" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="Q57" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="B58">
         <v>59</v>
       </c>
       <c r="Q58" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="B59">
         <v>73</v>
       </c>
       <c r="Q59" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>390</v>
+        <v>376</v>
       </c>
       <c r="B60">
         <v>45</v>
       </c>
       <c r="Q60" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Terminal Pesqueiro: Troca seaborn por plotly
</commit_message>
<xml_diff>
--- a/data/tabela_combinada_final.xlsx
+++ b/data/tabela_combinada_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\OneDrive\Documentos\D.comercial\dashboard streamlit\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC35640-23F6-4E47-A92D-2076D7937882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6AA21BF-970D-42EB-9294-023F3417DC3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="370">
   <si>
     <t>Nome do Participante</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Adagilson Nazaré Bezerra</t>
   </si>
   <si>
-    <t>Revenda, comerciantes</t>
-  </si>
-  <si>
     <t>Canoa, rede, manzuá</t>
   </si>
   <si>
@@ -123,9 +120,6 @@
     <t>Antonio Alves dos Santos</t>
   </si>
   <si>
-    <t>Diversos comerciantes</t>
-  </si>
-  <si>
     <t>Canoa, espinhal, rede</t>
   </si>
   <si>
@@ -165,9 +159,6 @@
     <t>Antônio Carlos Borges</t>
   </si>
   <si>
-    <t>Peixeiro (Silvério)</t>
-  </si>
-  <si>
     <t>Canoa, Rede</t>
   </si>
   <si>
@@ -204,9 +195,6 @@
     <t>Francisco de Assis Fernandes Ferreira</t>
   </si>
   <si>
-    <t>Comerciante</t>
-  </si>
-  <si>
     <t>Canoa, Artesanal</t>
   </si>
   <si>
@@ -237,9 +225,6 @@
     <t>Itamar Edson de Lima</t>
   </si>
   <si>
-    <t>Machante</t>
-  </si>
-  <si>
     <t>Sardinha</t>
   </si>
   <si>
@@ -267,9 +252,6 @@
     <t>José Cosmo Neto</t>
   </si>
   <si>
-    <t>Moto boy, Dono da Câmara Frigorífica</t>
-  </si>
-  <si>
     <t>Anzol, Rede, Canoa</t>
   </si>
   <si>
@@ -303,9 +285,6 @@
     <t>Paulo Eurico do Nascimento</t>
   </si>
   <si>
-    <t>Comerciantes, revenda</t>
-  </si>
-  <si>
     <t>Balsa, rede</t>
   </si>
   <si>
@@ -363,9 +342,6 @@
     <t>Antonio Carlos de Lima Pereira</t>
   </si>
   <si>
-    <t>Consumidor</t>
-  </si>
-  <si>
     <t>Tarrafa, linha</t>
   </si>
   <si>
@@ -429,9 +405,6 @@
     <t>Antonio Santos Sousa</t>
   </si>
   <si>
-    <t>Consumidor direto, comerciantes</t>
-  </si>
-  <si>
     <t>Canoa, isca, rede e tarrafa</t>
   </si>
   <si>
@@ -858,9 +831,6 @@
     <t>Charles Pereira de Lima</t>
   </si>
   <si>
-    <t>Vendem na rua a pé ou bicicleta</t>
-  </si>
-  <si>
     <t>Caçoeira</t>
   </si>
   <si>
@@ -1014,9 +984,6 @@
     <t>Paulo Iran Araújo Falcão</t>
   </si>
   <si>
-    <t>Coloca no grupo de WhatsApp e o comprador aciona ele (litoral pesca)</t>
-  </si>
-  <si>
     <t>Às vezes, depdente da maré</t>
   </si>
   <si>
@@ -1096,9 +1063,6 @@
   </si>
   <si>
     <t>Jarley Platini Galeno de Souza</t>
-  </si>
-  <si>
-    <t>População</t>
   </si>
   <si>
     <t>Sim, dentro do rio</t>
@@ -1616,2856 +1580,2856 @@
         <v>45</v>
       </c>
       <c r="C2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>24</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
+        <v>365</v>
+      </c>
+      <c r="O2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" t="s">
         <v>28</v>
       </c>
-      <c r="N2" t="s">
-        <v>377</v>
-      </c>
-      <c r="O2" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>29</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>66</v>
       </c>
       <c r="C3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
         <v>32</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>33</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>34</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>36</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>37</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>38</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>39</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>40</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
+        <v>366</v>
+      </c>
+      <c r="O3" t="s">
         <v>41</v>
       </c>
-      <c r="M3" t="s">
+      <c r="P3" t="s">
         <v>42</v>
       </c>
-      <c r="N3" t="s">
-        <v>378</v>
-      </c>
-      <c r="O3" t="s">
-        <v>43</v>
-      </c>
-      <c r="P3" t="s">
-        <v>44</v>
-      </c>
       <c r="Q3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4">
         <v>65</v>
       </c>
       <c r="C4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
         <v>46</v>
       </c>
-      <c r="D4" t="s">
+      <c r="H4" t="s">
         <v>47</v>
       </c>
-      <c r="E4" t="s">
+      <c r="I4" t="s">
         <v>48</v>
       </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="J4" t="s">
         <v>49</v>
       </c>
-      <c r="H4" t="s">
+      <c r="K4" t="s">
         <v>50</v>
       </c>
-      <c r="I4" t="s">
+      <c r="L4" t="s">
         <v>51</v>
       </c>
-      <c r="J4" t="s">
+      <c r="M4" t="s">
         <v>52</v>
       </c>
-      <c r="K4" t="s">
+      <c r="N4" t="s">
+        <v>42</v>
+      </c>
+      <c r="O4" t="s">
         <v>53</v>
       </c>
-      <c r="L4" t="s">
+      <c r="P4" t="s">
         <v>54</v>
       </c>
-      <c r="M4" t="s">
-        <v>55</v>
-      </c>
-      <c r="N4" t="s">
-        <v>44</v>
-      </c>
-      <c r="O4" t="s">
-        <v>56</v>
-      </c>
-      <c r="P4" t="s">
-        <v>57</v>
-      </c>
       <c r="Q4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B5">
         <v>54</v>
       </c>
       <c r="C5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" t="s">
         <v>59</v>
       </c>
-      <c r="D5" t="s">
+      <c r="J5" t="s">
         <v>60</v>
       </c>
-      <c r="E5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="K5" t="s">
         <v>61</v>
       </c>
-      <c r="H5" t="s">
+      <c r="L5" t="s">
         <v>62</v>
       </c>
-      <c r="I5" t="s">
+      <c r="M5" t="s">
         <v>63</v>
       </c>
-      <c r="J5" t="s">
+      <c r="N5" t="s">
+        <v>42</v>
+      </c>
+      <c r="O5" t="s">
         <v>64</v>
       </c>
-      <c r="K5" t="s">
-        <v>65</v>
-      </c>
-      <c r="L5" t="s">
-        <v>66</v>
-      </c>
-      <c r="M5" t="s">
-        <v>67</v>
-      </c>
-      <c r="N5" t="s">
-        <v>44</v>
-      </c>
-      <c r="O5" t="s">
-        <v>68</v>
-      </c>
       <c r="P5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B6">
         <v>62</v>
       </c>
       <c r="C6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K6" t="s">
         <v>70</v>
       </c>
-      <c r="D6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="L6" t="s">
         <v>71</v>
       </c>
-      <c r="F6" t="s">
+      <c r="M6" t="s">
         <v>72</v>
       </c>
-      <c r="G6" t="s">
+      <c r="N6" t="s">
+        <v>42</v>
+      </c>
+      <c r="O6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" t="s">
-        <v>74</v>
-      </c>
-      <c r="K6" t="s">
-        <v>75</v>
-      </c>
-      <c r="L6" t="s">
-        <v>76</v>
-      </c>
-      <c r="M6" t="s">
-        <v>77</v>
-      </c>
-      <c r="N6" t="s">
-        <v>44</v>
-      </c>
-      <c r="O6" t="s">
-        <v>78</v>
-      </c>
       <c r="P6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B7">
         <v>71</v>
       </c>
       <c r="C7" t="s">
+        <v>150</v>
+      </c>
+      <c r="D7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>78</v>
+      </c>
+      <c r="I7" t="s">
+        <v>79</v>
+      </c>
+      <c r="J7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" t="s">
         <v>80</v>
       </c>
-      <c r="D7" t="s">
+      <c r="L7" t="s">
         <v>81</v>
       </c>
-      <c r="E7" t="s">
+      <c r="M7" t="s">
         <v>82</v>
       </c>
-      <c r="F7" t="s">
+      <c r="N7" t="s">
+        <v>366</v>
+      </c>
+      <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="G7" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="P7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" t="s">
-        <v>85</v>
-      </c>
-      <c r="J7" t="s">
-        <v>25</v>
-      </c>
-      <c r="K7" t="s">
-        <v>86</v>
-      </c>
-      <c r="L7" t="s">
-        <v>87</v>
-      </c>
-      <c r="M7" t="s">
-        <v>88</v>
-      </c>
-      <c r="N7" t="s">
-        <v>378</v>
-      </c>
-      <c r="O7" t="s">
-        <v>89</v>
-      </c>
-      <c r="P7" t="s">
-        <v>90</v>
-      </c>
       <c r="Q7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B8">
         <v>29</v>
       </c>
       <c r="C8" t="s">
+        <v>150</v>
+      </c>
+      <c r="D8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" t="s">
+        <v>88</v>
+      </c>
+      <c r="K8" t="s">
+        <v>89</v>
+      </c>
+      <c r="L8" t="s">
+        <v>90</v>
+      </c>
+      <c r="M8" t="s">
+        <v>91</v>
+      </c>
+      <c r="N8" t="s">
+        <v>365</v>
+      </c>
+      <c r="O8" t="s">
         <v>92</v>
       </c>
-      <c r="D8" t="s">
-        <v>93</v>
-      </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>94</v>
-      </c>
-      <c r="H8" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" t="s">
-        <v>24</v>
-      </c>
-      <c r="J8" t="s">
-        <v>95</v>
-      </c>
-      <c r="K8" t="s">
-        <v>96</v>
-      </c>
-      <c r="L8" t="s">
-        <v>97</v>
-      </c>
-      <c r="M8" t="s">
-        <v>98</v>
-      </c>
-      <c r="N8" t="s">
-        <v>377</v>
-      </c>
-      <c r="O8" t="s">
-        <v>99</v>
-      </c>
       <c r="P8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B9">
         <v>50</v>
       </c>
       <c r="C9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" t="s">
+        <v>96</v>
+      </c>
+      <c r="H9" t="s">
+        <v>97</v>
+      </c>
+      <c r="I9" t="s">
+        <v>98</v>
+      </c>
+      <c r="J9" t="s">
+        <v>99</v>
+      </c>
+      <c r="K9" t="s">
+        <v>100</v>
+      </c>
+      <c r="L9" t="s">
         <v>101</v>
       </c>
-      <c r="D9" t="s">
+      <c r="M9" t="s">
         <v>102</v>
       </c>
-      <c r="E9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="N9" t="s">
+        <v>42</v>
+      </c>
+      <c r="O9" t="s">
         <v>103</v>
       </c>
-      <c r="H9" t="s">
-        <v>104</v>
-      </c>
-      <c r="I9" t="s">
-        <v>105</v>
-      </c>
-      <c r="J9" t="s">
-        <v>106</v>
-      </c>
-      <c r="K9" t="s">
-        <v>107</v>
-      </c>
-      <c r="L9" t="s">
-        <v>108</v>
-      </c>
-      <c r="M9" t="s">
-        <v>109</v>
-      </c>
-      <c r="N9" t="s">
-        <v>44</v>
-      </c>
-      <c r="O9" t="s">
-        <v>110</v>
-      </c>
       <c r="P9" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B10">
         <v>58</v>
       </c>
       <c r="C10" t="s">
+        <v>247</v>
+      </c>
+      <c r="D10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" t="s">
+        <v>107</v>
+      </c>
+      <c r="G10" t="s">
+        <v>108</v>
+      </c>
+      <c r="H10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I10" t="s">
+        <v>110</v>
+      </c>
+      <c r="J10" t="s">
+        <v>111</v>
+      </c>
+      <c r="K10" t="s">
         <v>112</v>
       </c>
-      <c r="D10" t="s">
+      <c r="L10" t="s">
         <v>113</v>
       </c>
-      <c r="E10" t="s">
+      <c r="M10" t="s">
         <v>114</v>
       </c>
-      <c r="F10" t="s">
+      <c r="N10" t="s">
+        <v>365</v>
+      </c>
+      <c r="O10" t="s">
         <v>115</v>
       </c>
-      <c r="G10" t="s">
+      <c r="P10" t="s">
         <v>116</v>
       </c>
-      <c r="H10" t="s">
+      <c r="Q10" t="s">
         <v>117</v>
-      </c>
-      <c r="I10" t="s">
-        <v>118</v>
-      </c>
-      <c r="J10" t="s">
-        <v>119</v>
-      </c>
-      <c r="K10" t="s">
-        <v>120</v>
-      </c>
-      <c r="L10" t="s">
-        <v>121</v>
-      </c>
-      <c r="M10" t="s">
-        <v>122</v>
-      </c>
-      <c r="N10" t="s">
-        <v>377</v>
-      </c>
-      <c r="O10" t="s">
-        <v>123</v>
-      </c>
-      <c r="P10" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B11">
         <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F11" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G11" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="H11" t="s">
+        <v>109</v>
+      </c>
+      <c r="I11" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" t="s">
+        <v>122</v>
+      </c>
+      <c r="K11" t="s">
+        <v>121</v>
+      </c>
+      <c r="L11" t="s">
+        <v>111</v>
+      </c>
+      <c r="M11" t="s">
+        <v>123</v>
+      </c>
+      <c r="N11" t="s">
+        <v>366</v>
+      </c>
+      <c r="O11" t="s">
+        <v>124</v>
+      </c>
+      <c r="P11" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q11" t="s">
         <v>117</v>
-      </c>
-      <c r="I11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J11" t="s">
-        <v>130</v>
-      </c>
-      <c r="K11" t="s">
-        <v>129</v>
-      </c>
-      <c r="L11" t="s">
-        <v>119</v>
-      </c>
-      <c r="M11" t="s">
-        <v>131</v>
-      </c>
-      <c r="N11" t="s">
-        <v>378</v>
-      </c>
-      <c r="O11" t="s">
-        <v>132</v>
-      </c>
-      <c r="P11" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="B12">
         <v>55</v>
       </c>
       <c r="C12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" t="s">
+        <v>120</v>
+      </c>
+      <c r="F12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12" t="s">
+        <v>128</v>
+      </c>
+      <c r="H12" t="s">
+        <v>129</v>
+      </c>
+      <c r="I12" t="s">
+        <v>110</v>
+      </c>
+      <c r="J12" t="s">
+        <v>130</v>
+      </c>
+      <c r="K12" t="s">
+        <v>131</v>
+      </c>
+      <c r="L12" t="s">
+        <v>132</v>
+      </c>
+      <c r="M12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N12" t="s">
+        <v>367</v>
+      </c>
+      <c r="O12" t="s">
         <v>134</v>
       </c>
-      <c r="D12" t="s">
-        <v>135</v>
-      </c>
-      <c r="E12" t="s">
-        <v>128</v>
-      </c>
-      <c r="F12" t="s">
-        <v>136</v>
-      </c>
-      <c r="G12" t="s">
-        <v>137</v>
-      </c>
-      <c r="H12" t="s">
-        <v>138</v>
-      </c>
-      <c r="I12" t="s">
-        <v>118</v>
-      </c>
-      <c r="J12" t="s">
-        <v>139</v>
-      </c>
-      <c r="K12" t="s">
-        <v>140</v>
-      </c>
-      <c r="L12" t="s">
-        <v>141</v>
-      </c>
-      <c r="M12" t="s">
-        <v>142</v>
-      </c>
-      <c r="N12" t="s">
-        <v>379</v>
-      </c>
-      <c r="O12" t="s">
-        <v>143</v>
-      </c>
       <c r="P12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q12" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B13">
         <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D13" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E13" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F13" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G13" t="s">
+        <v>121</v>
+      </c>
+      <c r="H13" t="s">
         <v>129</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
+        <v>137</v>
+      </c>
+      <c r="J13" t="s">
+        <v>62</v>
+      </c>
+      <c r="K13" t="s">
         <v>138</v>
       </c>
-      <c r="I13" t="s">
-        <v>146</v>
-      </c>
-      <c r="J13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K13" t="s">
-        <v>147</v>
-      </c>
       <c r="L13" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="M13" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="N13" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O13" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="P13" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q13" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="B14">
         <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H14" t="s">
+        <v>129</v>
+      </c>
+      <c r="I14" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" t="s">
+        <v>62</v>
+      </c>
+      <c r="K14" t="s">
+        <v>121</v>
+      </c>
+      <c r="L14" t="s">
+        <v>143</v>
+      </c>
+      <c r="M14" t="s">
+        <v>144</v>
+      </c>
+      <c r="N14" t="s">
+        <v>365</v>
+      </c>
+      <c r="O14" t="s">
         <v>145</v>
       </c>
-      <c r="E14" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" t="s">
-        <v>129</v>
-      </c>
-      <c r="H14" t="s">
-        <v>138</v>
-      </c>
-      <c r="I14" t="s">
-        <v>24</v>
-      </c>
-      <c r="J14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K14" t="s">
-        <v>129</v>
-      </c>
-      <c r="L14" t="s">
-        <v>152</v>
-      </c>
-      <c r="M14" t="s">
-        <v>153</v>
-      </c>
-      <c r="N14" t="s">
-        <v>377</v>
-      </c>
-      <c r="O14" t="s">
-        <v>154</v>
-      </c>
       <c r="P14" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q14" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="B15">
         <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D15" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" t="s">
+        <v>129</v>
+      </c>
+      <c r="I15" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" t="s">
+        <v>147</v>
+      </c>
+      <c r="K15" t="s">
+        <v>148</v>
+      </c>
+      <c r="L15" t="s">
+        <v>39</v>
+      </c>
+      <c r="M15" t="s">
+        <v>140</v>
+      </c>
+      <c r="N15" t="s">
+        <v>365</v>
+      </c>
+      <c r="O15" t="s">
         <v>145</v>
       </c>
-      <c r="E15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F15" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" t="s">
-        <v>44</v>
-      </c>
-      <c r="H15" t="s">
-        <v>138</v>
-      </c>
-      <c r="I15" t="s">
-        <v>51</v>
-      </c>
-      <c r="J15" t="s">
-        <v>156</v>
-      </c>
-      <c r="K15" t="s">
-        <v>157</v>
-      </c>
-      <c r="L15" t="s">
-        <v>41</v>
-      </c>
-      <c r="M15" t="s">
-        <v>149</v>
-      </c>
-      <c r="N15" t="s">
-        <v>377</v>
-      </c>
-      <c r="O15" t="s">
-        <v>154</v>
-      </c>
       <c r="P15" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q15" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B16">
         <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D16" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E16" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="H16" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I16" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="J16" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K16" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="L16" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="M16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="N16" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O16" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="P16" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q16" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="B17">
         <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D17" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="E17" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F17" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G17" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="H17" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I17" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="J17" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K17" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L17" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M17" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="N17" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O17" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="P17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q17" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B18">
         <v>60</v>
       </c>
       <c r="C18" t="s">
+        <v>156</v>
+      </c>
+      <c r="D18" t="s">
+        <v>164</v>
+      </c>
+      <c r="E18" t="s">
         <v>165</v>
       </c>
-      <c r="D18" t="s">
-        <v>173</v>
-      </c>
-      <c r="E18" t="s">
-        <v>174</v>
-      </c>
       <c r="F18" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G18" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="H18" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J18" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K18" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="L18" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M18" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="N18" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O18" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="P18" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q18" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="B19">
         <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D19" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G19" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="H19" t="s">
+        <v>109</v>
+      </c>
+      <c r="I19" t="s">
+        <v>170</v>
+      </c>
+      <c r="J19" t="s">
+        <v>171</v>
+      </c>
+      <c r="K19" t="s">
+        <v>121</v>
+      </c>
+      <c r="L19" t="s">
+        <v>143</v>
+      </c>
+      <c r="M19" t="s">
+        <v>140</v>
+      </c>
+      <c r="N19" t="s">
+        <v>366</v>
+      </c>
+      <c r="O19" t="s">
+        <v>172</v>
+      </c>
+      <c r="P19" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q19" t="s">
         <v>117</v>
-      </c>
-      <c r="I19" t="s">
-        <v>179</v>
-      </c>
-      <c r="J19" t="s">
-        <v>180</v>
-      </c>
-      <c r="K19" t="s">
-        <v>129</v>
-      </c>
-      <c r="L19" t="s">
-        <v>152</v>
-      </c>
-      <c r="M19" t="s">
-        <v>149</v>
-      </c>
-      <c r="N19" t="s">
-        <v>378</v>
-      </c>
-      <c r="O19" t="s">
-        <v>181</v>
-      </c>
-      <c r="P19" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="B20">
         <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D20" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="E20" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="F20" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="G20" t="s">
+        <v>121</v>
+      </c>
+      <c r="H20" t="s">
         <v>129</v>
       </c>
-      <c r="H20" t="s">
-        <v>138</v>
-      </c>
       <c r="I20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" t="s">
         <v>24</v>
       </c>
-      <c r="J20" t="s">
-        <v>25</v>
-      </c>
       <c r="K20" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="L20" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M20" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="N20" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O20" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="P20" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q20" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="B21">
         <v>40</v>
       </c>
       <c r="C21" t="s">
+        <v>156</v>
+      </c>
+      <c r="D21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E21" t="s">
         <v>165</v>
       </c>
-      <c r="D21" t="s">
-        <v>187</v>
-      </c>
-      <c r="E21" t="s">
-        <v>174</v>
-      </c>
       <c r="F21" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="G21" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="H21" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K21" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="L21" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="M21" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="N21" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O21" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="P21" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q21" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B22">
         <v>56</v>
       </c>
       <c r="C22" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D22" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G22" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="H22" t="s">
+        <v>109</v>
+      </c>
+      <c r="I22" t="s">
+        <v>59</v>
+      </c>
+      <c r="J22" t="s">
+        <v>186</v>
+      </c>
+      <c r="K22" t="s">
+        <v>148</v>
+      </c>
+      <c r="L22" t="s">
+        <v>71</v>
+      </c>
+      <c r="M22" t="s">
+        <v>102</v>
+      </c>
+      <c r="N22" t="s">
+        <v>366</v>
+      </c>
+      <c r="O22" t="s">
+        <v>187</v>
+      </c>
+      <c r="P22" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q22" t="s">
         <v>117</v>
-      </c>
-      <c r="I22" t="s">
-        <v>63</v>
-      </c>
-      <c r="J22" t="s">
-        <v>195</v>
-      </c>
-      <c r="K22" t="s">
-        <v>157</v>
-      </c>
-      <c r="L22" t="s">
-        <v>76</v>
-      </c>
-      <c r="M22" t="s">
-        <v>109</v>
-      </c>
-      <c r="N22" t="s">
-        <v>378</v>
-      </c>
-      <c r="O22" t="s">
-        <v>196</v>
-      </c>
-      <c r="P22" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B23">
         <v>62</v>
       </c>
       <c r="C23" t="s">
-        <v>134</v>
+        <v>247</v>
       </c>
       <c r="D23" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="E23" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F23" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G23" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="H23" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I23" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="J23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K23" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="L23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M23" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="N23" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O23" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="P23" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q23" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B24">
         <v>63</v>
       </c>
       <c r="C24" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D24" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="E24" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="F24" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="G24" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="H24" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I24" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J24" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="K24" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="L24" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="M24" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="N24" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O24" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="P24" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q24" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B25">
         <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D25" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E25" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="F25" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G25" t="s">
+        <v>121</v>
+      </c>
+      <c r="H25" t="s">
         <v>129</v>
       </c>
-      <c r="H25" t="s">
-        <v>138</v>
-      </c>
       <c r="I25" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="J25" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="K25" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="L25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M25" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="N25" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O25" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="P25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q25" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B26">
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="D26" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="E26" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="F26" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G26" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="H26" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J26" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="K26" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="L26" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="M26" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="N26" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="O26" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="P26" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q26" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B27">
         <v>53</v>
       </c>
       <c r="C27" t="s">
-        <v>112</v>
+        <v>247</v>
       </c>
       <c r="D27" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="E27" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F27" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G27" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="H27" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I27" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="J27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K27" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="L27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M27" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="N27" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O27" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="P27" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q27" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B28">
         <v>51</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D28" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G28" t="s">
+        <v>121</v>
+      </c>
+      <c r="H28" t="s">
         <v>129</v>
       </c>
-      <c r="H28" t="s">
-        <v>138</v>
-      </c>
       <c r="I28" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="J28" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="K28" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L28" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="M28" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="N28" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O28" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="P28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q28" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="B29">
         <v>49</v>
       </c>
       <c r="C29" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D29" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="E29" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="F29" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="G29" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="H29" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I29" t="s">
+        <v>223</v>
+      </c>
+      <c r="J29" t="s">
+        <v>230</v>
+      </c>
+      <c r="K29" t="s">
+        <v>231</v>
+      </c>
+      <c r="L29" t="s">
+        <v>224</v>
+      </c>
+      <c r="M29" t="s">
         <v>232</v>
       </c>
-      <c r="J29" t="s">
-        <v>239</v>
-      </c>
-      <c r="K29" t="s">
-        <v>240</v>
-      </c>
-      <c r="L29" t="s">
+      <c r="N29" t="s">
+        <v>366</v>
+      </c>
+      <c r="O29" t="s">
         <v>233</v>
       </c>
-      <c r="M29" t="s">
-        <v>241</v>
-      </c>
-      <c r="N29" t="s">
-        <v>378</v>
-      </c>
-      <c r="O29" t="s">
-        <v>242</v>
-      </c>
       <c r="P29" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="Q29" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B30">
         <v>74</v>
       </c>
       <c r="C30" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="D30" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="E30" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="F30" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G30" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="H30" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I30" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="J30" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="K30" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="L30" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="M30" t="s">
+        <v>232</v>
+      </c>
+      <c r="N30" t="s">
+        <v>366</v>
+      </c>
+      <c r="O30" t="s">
         <v>241</v>
       </c>
-      <c r="N30" t="s">
-        <v>378</v>
-      </c>
-      <c r="O30" t="s">
-        <v>250</v>
-      </c>
       <c r="P30" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q30" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="B31">
         <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D31" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E31" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G31" t="s">
+        <v>121</v>
+      </c>
+      <c r="H31" t="s">
         <v>129</v>
       </c>
-      <c r="H31" t="s">
-        <v>138</v>
-      </c>
       <c r="I31" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="J31" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="K31" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="L31" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="M31" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="N31" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O31" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="P31" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q31" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="B32">
         <v>57</v>
       </c>
       <c r="C32" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D32" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E32" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G32" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="H32" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I32" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="J32" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="K32" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="L32" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="M32" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="O32" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="P32" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q32" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B33">
         <v>37</v>
       </c>
       <c r="C33" t="s">
+        <v>247</v>
+      </c>
+      <c r="D33" t="s">
+        <v>254</v>
+      </c>
+      <c r="E33" t="s">
         <v>165</v>
       </c>
-      <c r="D33" t="s">
-        <v>263</v>
-      </c>
-      <c r="E33" t="s">
-        <v>174</v>
-      </c>
       <c r="F33" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="G33" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="H33" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I33" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="J33" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="K33" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="L33" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="M33" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="N33" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O33" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="P33" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q33" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="B34">
         <v>30</v>
       </c>
       <c r="C34" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F34" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="G34" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H34" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I34" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K34" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L34" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="M34" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="N34" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O34" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="P34" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q34" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="B35">
         <v>44</v>
       </c>
       <c r="C35" t="s">
-        <v>277</v>
+        <v>247</v>
       </c>
       <c r="D35" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="E35" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G35" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H35" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J35" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K35" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L35" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M35" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="N35" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="O35" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="P35" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="Q35" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="B36">
         <v>56</v>
       </c>
       <c r="C36" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D36" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="E36" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="F36" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G36" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H36" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I36" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K36" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="L36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M36" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="N36" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O36" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="P36" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="Q36" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="B37">
         <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D37" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="E37" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="F37" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G37" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H37" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I37" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J37" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K37" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="L37" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M37" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="N37" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O37" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="P37" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="Q37" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="C38" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D38" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="E38" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="F38" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H38" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I38" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J38" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K38" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="L38" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M38" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="N38" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O38" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="P38" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="Q38" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="B39">
         <v>34</v>
       </c>
       <c r="Q39" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="B40">
         <v>73</v>
       </c>
       <c r="Q40" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="B41">
         <v>44</v>
       </c>
       <c r="C41" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="E41" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="F41" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="G41" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="H41" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I41" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J41" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="K41" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="L41" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="M41" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="N41" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O41" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="P41" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q41" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="B42">
         <v>52</v>
       </c>
       <c r="C42" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D42" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E42" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F42" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G42" t="s">
+        <v>121</v>
+      </c>
+      <c r="H42" t="s">
         <v>129</v>
       </c>
-      <c r="H42" t="s">
-        <v>138</v>
-      </c>
       <c r="I42" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="J42" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="K42" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L42" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M42" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="N42" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O42" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="P42" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q42" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="B43">
         <v>45</v>
       </c>
       <c r="C43" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D43" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="E43" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F43" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="G43" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="H43" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I43" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="J43" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="K43" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L43" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="M43" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="N43" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O43" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="P43" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q43" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="B44">
         <v>32</v>
       </c>
       <c r="C44" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D44" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="E44" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="F44" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="G44" t="s">
+        <v>121</v>
+      </c>
+      <c r="H44" t="s">
         <v>129</v>
       </c>
-      <c r="H44" t="s">
-        <v>138</v>
-      </c>
       <c r="I44" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J44" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K44" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="L44" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M44" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="N44" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="O44" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="P44" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q44" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="B45">
         <v>26</v>
       </c>
       <c r="C45" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D45" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="E45" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="F45" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="G45" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="H45" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I45" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J45" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="K45" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="L45" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="M45" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="N45" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O45" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="P45" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q45" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="B46">
         <v>55</v>
       </c>
       <c r="C46" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D46" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="E46" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F46" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="G46" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="H46" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I46" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="J46" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="K46" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L46" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="M46" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="N46" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O46" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="P46" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q46" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="B47">
         <v>51</v>
       </c>
       <c r="C47" t="s">
-        <v>329</v>
+        <v>261</v>
       </c>
       <c r="D47" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="E47" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="F47" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G47" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="H47" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J47" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="K47" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L47" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="M47" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="N47" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O47" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="P47" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q47" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="B48">
         <v>41</v>
       </c>
       <c r="C48" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D48" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="E48" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="F48" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G48" t="s">
+        <v>314</v>
+      </c>
+      <c r="H48" t="s">
+        <v>129</v>
+      </c>
+      <c r="I48" t="s">
+        <v>323</v>
+      </c>
+      <c r="J48" t="s">
+        <v>197</v>
+      </c>
+      <c r="K48" t="s">
+        <v>68</v>
+      </c>
+      <c r="L48" t="s">
         <v>324</v>
       </c>
-      <c r="H48" t="s">
-        <v>138</v>
-      </c>
-      <c r="I48" t="s">
-        <v>334</v>
-      </c>
-      <c r="J48" t="s">
-        <v>206</v>
-      </c>
-      <c r="K48" t="s">
-        <v>73</v>
-      </c>
-      <c r="L48" t="s">
-        <v>335</v>
-      </c>
       <c r="M48" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="N48" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="O48" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="P48" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="Q48" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="B49">
         <v>45</v>
       </c>
       <c r="C49" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D49" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="E49" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F49" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="G49" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="H49" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I49" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="J49" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="K49" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L49" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="M49" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="N49" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O49" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="P49" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="Q49" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="B50">
         <v>53</v>
       </c>
       <c r="C50" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D50" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="E50" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="F50" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G50" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="H50" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I50" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="J50" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K50" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
       <c r="L50" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="M50" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="O50" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
       <c r="P50" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q50" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>347</v>
+        <v>336</v>
       </c>
       <c r="B51">
         <v>32</v>
       </c>
       <c r="C51" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D51" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G51" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="H51" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
       <c r="I51" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="J51" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="K51" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="L51" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="M51" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="O51" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="P51" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q51" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="B52">
         <v>54</v>
       </c>
       <c r="C52" t="s">
-        <v>59</v>
+        <v>150</v>
       </c>
       <c r="D52" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
       <c r="G52" t="s">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="H52" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I52" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="J52" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K52" t="s">
-        <v>354</v>
+        <v>343</v>
       </c>
       <c r="L52" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M52" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="N52" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O52" t="s">
-        <v>355</v>
+        <v>344</v>
       </c>
       <c r="P52" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q52" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="B53">
         <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>357</v>
+        <v>247</v>
       </c>
       <c r="D53" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G53" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="H53" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="J53" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K53" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="L53" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M53" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="N53" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O53" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="P53" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="Q53" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="B54">
         <v>63</v>
       </c>
       <c r="C54" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D54" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G54" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H54" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I54" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="J54" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L54" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="M54" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="N54" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="O54" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="P54" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="Q54" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="B55">
         <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D55" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G55" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="H55" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="J55" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K55" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="L55" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M55" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="N55" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="O55" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="P55" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q55" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="B56">
         <v>41</v>
       </c>
       <c r="C56" t="s">
-        <v>357</v>
+        <v>247</v>
       </c>
       <c r="D56" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G56" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="H56" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="I56" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="J56" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K56" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="L56" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M56" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="N56" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O56" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="P56" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="Q56" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="B57">
         <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D57" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="E57" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="F57" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G57" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="H57" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="J57" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="K57" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="L57" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="M57" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="N57" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="O57" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="P57" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="Q57" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="B58">
         <v>59</v>
       </c>
       <c r="Q58" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="B59">
         <v>73</v>
       </c>
       <c r="Q59" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="B60">
         <v>45</v>
       </c>
       <c r="Q60" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TP: adiçao novos graficos
</commit_message>
<xml_diff>
--- a/data/tabela_combinada_final.xlsx
+++ b/data/tabela_combinada_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\OneDrive\Documentos\D.comercial\dashboard streamlit\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6AA21BF-970D-42EB-9294-023F3417DC3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D62568D-3F6A-4B7F-BD9A-232555FF36CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="369">
   <si>
     <t>Nome do Participante</t>
   </si>
@@ -1132,9 +1132,6 @@
   </si>
   <si>
     <t>lua cheia</t>
-  </si>
-  <si>
-    <t>lua escura</t>
   </si>
 </sst>
 </file>
@@ -3961,7 +3958,7 @@
         <v>325</v>
       </c>
       <c r="N48" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="O48" t="s">
         <v>326</v>

</xml_diff>